<commit_message>
feat(johto): add Diglett Cave to map coordinates and re-export excel
- Added the requested Diglett Cave map spot to config/johtoMapCoordinates.js
- Regenerated the 2_Johto_Data.xlsx file so that Diglett Cave will show "1" in the Map column.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2_Johto_Data.xlsx
+++ b/2_Johto_Data.xlsx
@@ -4539,7 +4539,7 @@
         <v>90%</v>
       </c>
       <c r="G180">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="181">
@@ -4562,7 +4562,7 @@
         <v>10%</v>
       </c>
       <c r="G181">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -8184,7 +8184,7 @@
         <v>Diglett Cave</v>
       </c>
       <c r="C38">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39">

</xml_diff>